<commit_message>
Update pages with global loader
</commit_message>
<xml_diff>
--- a/excel_routes/route_MED_ATZ_threats.xlsx
+++ b/excel_routes/route_MED_ATZ_threats.xlsx
@@ -523,24 +523,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>21-JUN-26</t>
+          <t>23-JUN-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM-252</t>
+          <t>SM-254</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-101</t>
+          <t>EgyptAir MS-103</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1550</v>
+        <v>1650</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1730</v>
+        <v>1790</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>-200</v>

</xml_diff>